<commit_message>
Hoàn thành 7 biểu đồ còn thiếu, kiểm chất lượng dữ liệu và trang web
Biểu đồ mới (T09, T15, T16, T17, T19, T20, T21):
- phân bố bậc log-log: bác bỏ giả định mạng scale-free
- node-link và hai ma trận kề trên CÙNG 416 cạnh, để so hai họ biểu diễn
- chord 10 khối, Việt Nam tách riêng làm trọng tâm
- Sankey nhập/xuất, small multiples theo thời gian, streamgraph 10 ngành

T08 đổi hướng: Atlas và BACI đều dẫn xuất từ Comtrade nên không phải ba nguồn
độc lập. Thay bằng chênh lệch gương ngay trong dữ liệu. Kết quả 2093/2093 luồng
trùng khít, tức Atlas đã hòa giải số liệu và ta không tự đo được sai số của nó.

Cộng đồng mã hóa bằng ba nấc xám và ba hình dạng, không bằng màu: đã đo 7 bảng
3 màu ứng viên, bảng nào cũng tụt xuống ΔE 2,6-6,6 so với màu ngành gần nhất
khi mô phỏng mù màu.

Thêm docs/ket-luan-cho-thuyet-trinh.md, phuong-phap-luan.md (T25),
phat-hien.md (T26), cau-hoi-phan-bien.md (T29), và trang web tĩnh ở web/ (T27).
</commit_message>
<xml_diff>
--- a/phan-cong-cong-viec.xlsx
+++ b/phan-cong-cong-viec.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22188" windowHeight="9000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Phân công chi tiết" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hợp đồng dữ liệu" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tiến độ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Checklist nộp bài" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phân công chi tiết" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hợp đồng dữ liệu" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiến độ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist nộp bài" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Phân công chi tiết'!$A$4:$H$34</definedName>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2793,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Xong</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đang làm</t>
         </is>
       </c>
     </row>
@@ -2913,10 +2913,11 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-    </row>
+          <t>Đang làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
     <row r="36">
       <c r="B36" s="27" t="inlineStr">
         <is>

</xml_diff>